<commit_message>
chore: 新增 data 目錄
</commit_message>
<xml_diff>
--- a/data/興櫃的資料_updated.xlsx
+++ b/data/興櫃的資料_updated.xlsx
@@ -1,15 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xx8897\codespace\antigravity\台股文件\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{509155CD-DB77-4E63-84CD-15F41BC1BC7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -324,12 +335,6 @@
 (2024)股東獨享尊榮購物金2000元(可MAIL交付)</t>
   </si>
   <si>
-    <t>(2025)精緻衣物手洗精
-(2024)清淨海MIIFLORA清潔用品(隨機出貨)
-(2023)清淨海洗衣膠囊(18顆*8g)
-(2021)清潔用品(凱特的秘密)乙瓶</t>
-  </si>
-  <si>
     <t>(2025)7-11 100元商品卡</t>
   </si>
   <si>
@@ -338,16 +343,23 @@
 (2023)7-11商品卡35元
 (2022)超商商品卡100元</t>
   </si>
+  <si>
+    <t>(2025)精緻衣物手洗精
+(2024)清淨海MIIFLORA清潔用品
+(2023)清淨海洗衣膠囊(18顆*8g)
+(2021)清潔用品(凱特的秘密)乙瓶</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -355,8 +367,15 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -395,24 +414,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -450,7 +478,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -484,6 +512,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -518,9 +547,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -693,11 +723,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15.65" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -732,7 +762,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2758</v>
       </c>
@@ -751,11 +781,11 @@
       <c r="F2">
         <v>88</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>4132</v>
       </c>
@@ -777,11 +807,11 @@
       <c r="J3" t="s">
         <v>62</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4150</v>
       </c>
@@ -803,11 +833,11 @@
       <c r="J4" t="s">
         <v>62</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4172</v>
       </c>
@@ -829,11 +859,11 @@
       <c r="J5" t="s">
         <v>62</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4195</v>
       </c>
@@ -855,11 +885,11 @@
       <c r="J6" t="s">
         <v>62</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5262</v>
       </c>
@@ -881,11 +911,11 @@
       <c r="J7" t="s">
         <v>62</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>5863</v>
       </c>
@@ -907,11 +937,11 @@
       <c r="J8" t="s">
         <v>62</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6473</v>
       </c>
@@ -930,11 +960,11 @@
       <c r="F9">
         <v>7.87</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>6483</v>
       </c>
@@ -951,16 +981,16 @@
         <v>41</v>
       </c>
       <c r="F10">
-        <v>16.15</v>
+        <v>16.149999999999999</v>
       </c>
       <c r="J10" t="s">
         <v>62</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>6543</v>
       </c>
@@ -979,11 +1009,11 @@
       <c r="F11">
         <v>24.8</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>6549</v>
       </c>
@@ -1005,11 +1035,11 @@
       <c r="J12" t="s">
         <v>62</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>6586</v>
       </c>
@@ -1031,11 +1061,11 @@
       <c r="J13" t="s">
         <v>62</v>
       </c>
-      <c r="K13" t="s">
+      <c r="K13" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>6595</v>
       </c>
@@ -1052,16 +1082,16 @@
         <v>50</v>
       </c>
       <c r="F14">
-        <v>32.55</v>
+        <v>32.549999999999997</v>
       </c>
       <c r="J14" t="s">
         <v>62</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6618</v>
       </c>
@@ -1083,11 +1113,11 @@
       <c r="J15" t="s">
         <v>62</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>6621</v>
       </c>
@@ -1109,11 +1139,11 @@
       <c r="J16" t="s">
         <v>62</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>6648</v>
       </c>
@@ -1130,13 +1160,13 @@
         <v>51</v>
       </c>
       <c r="F17">
-        <v>17.85</v>
-      </c>
-      <c r="K17" t="s">
+        <v>17.850000000000001</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>6786</v>
       </c>
@@ -1153,16 +1183,16 @@
         <v>52</v>
       </c>
       <c r="F18">
-        <v>93.90000000000001</v>
+        <v>93.9</v>
       </c>
       <c r="J18" t="s">
         <v>62</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>6787</v>
       </c>
@@ -1184,11 +1214,11 @@
       <c r="J19" t="s">
         <v>62</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K19" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>6793</v>
       </c>
@@ -1210,11 +1240,11 @@
       <c r="J20" t="s">
         <v>62</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>6797</v>
       </c>
@@ -1236,11 +1266,11 @@
       <c r="J21" t="s">
         <v>62</v>
       </c>
-      <c r="K21" t="s">
+      <c r="K21" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>6798</v>
       </c>
@@ -1257,16 +1287,16 @@
         <v>55</v>
       </c>
       <c r="F22">
-        <v>38.8</v>
+        <v>38.799999999999997</v>
       </c>
       <c r="J22" t="s">
         <v>62</v>
       </c>
-      <c r="K22" t="s">
+      <c r="K22" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>6810</v>
       </c>
@@ -1288,11 +1318,11 @@
       <c r="J23" t="s">
         <v>62</v>
       </c>
-      <c r="K23" t="s">
+      <c r="K23" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>6815</v>
       </c>
@@ -1311,11 +1341,11 @@
       <c r="F24">
         <v>45.7</v>
       </c>
-      <c r="K24" t="s">
+      <c r="K24" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>6876</v>
       </c>
@@ -1337,11 +1367,11 @@
       <c r="J25" t="s">
         <v>62</v>
       </c>
-      <c r="K25" t="s">
+      <c r="K25" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>6886</v>
       </c>
@@ -1363,11 +1393,11 @@
       <c r="J26" t="s">
         <v>62</v>
       </c>
-      <c r="K26" t="s">
+      <c r="K26" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>7516</v>
       </c>
@@ -1384,16 +1414,16 @@
         <v>59</v>
       </c>
       <c r="F27">
-        <v>9.199999999999999</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="J27" t="s">
         <v>62</v>
       </c>
-      <c r="K27" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
+      <c r="K27" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>7566</v>
       </c>
@@ -1415,11 +1445,11 @@
       <c r="J28" t="s">
         <v>62</v>
       </c>
-      <c r="K28" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
+      <c r="K28" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>7719</v>
       </c>
@@ -1436,16 +1466,16 @@
         <v>41</v>
       </c>
       <c r="F29">
-        <v>38.2</v>
+        <v>38.200000000000003</v>
       </c>
       <c r="J29" t="s">
         <v>63</v>
       </c>
-      <c r="K29" t="s">
+      <c r="K29" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>8119</v>
       </c>
@@ -1468,10 +1498,11 @@
         <v>62</v>
       </c>
       <c r="K30" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>